<commit_message>
creating the list again, because, well, you always have to ask 16 times an ai to do something right
</commit_message>
<xml_diff>
--- a/documents/project_managment_tools/zoho_plan_comparaison.xlsx
+++ b/documents/project_managment_tools/zoho_plan_comparaison.xlsx
@@ -7,7 +7,7 @@
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Zoho Standalone Apps Overview" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="All Zoho Apps - Complete List" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -29,24 +29,19 @@
       <name val="Calibri"/>
       <b val="1"/>
       <color rgb="00FFFFFF"/>
-      <sz val="16"/>
+      <sz val="15"/>
     </font>
     <font>
       <name val="Calibri"/>
       <i val="1"/>
       <color rgb="00D9D9D9"/>
-      <sz val="11"/>
+      <sz val="10"/>
     </font>
     <font>
       <name val="Calibri"/>
       <b val="1"/>
       <color rgb="00FFFFFF"/>
       <sz val="11"/>
-    </font>
-    <font>
-      <name val="Calibri"/>
-      <color rgb="00333333"/>
-      <sz val="10"/>
     </font>
     <font>
       <name val="Calibri"/>
@@ -58,6 +53,11 @@
       <name val="Calibri"/>
       <b val="1"/>
       <color rgb="00000000"/>
+      <sz val="10"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <color rgb="00333333"/>
       <sz val="10"/>
     </font>
   </fonts>
@@ -130,22 +130,22 @@
     <xf numFmtId="0" fontId="3" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="4" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="5" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="top" wrapText="1"/>
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="6" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="4" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="top" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="6" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -513,27 +513,27 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E37"/>
+  <dimension ref="A1:E65"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="22" customWidth="1" min="1" max="1"/>
-    <col width="22" customWidth="1" min="2" max="2"/>
-    <col width="42" customWidth="1" min="3" max="3"/>
-    <col width="45" customWidth="1" min="4" max="4"/>
-    <col width="48" customWidth="1" min="5" max="5"/>
+    <col width="24" customWidth="1" min="1" max="1"/>
+    <col width="26" customWidth="1" min="2" max="2"/>
+    <col width="45" customWidth="1" min="3" max="3"/>
+    <col width="48" customWidth="1" min="4" max="4"/>
+    <col width="50" customWidth="1" min="5" max="5"/>
   </cols>
   <sheetData>
-    <row r="1" ht="30" customHeight="1">
+    <row r="1" ht="28" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>ZOHO STANDALONE APPLICATIONS: COMPREHENSIVE PLAN &amp; LIFECYCLE GUIDE</t>
-        </is>
-      </c>
-    </row>
-    <row r="2" ht="20" customHeight="1">
+          <t>COMPLETE ALL ZOHO APPS MASTER DIRECTORY (EVERY APP ON ITS OWN ROW)</t>
+        </is>
+      </c>
+    </row>
+    <row r="2" ht="18" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Complete breakdown of Free vs. Paid tiers, limitations, and trial expiration mechanics (Excluding Zoho One)</t>
+          <t>Every standalone Zoho application listed individually with explicit Free plan limits, Paid tier models, and post-trial/downgrade behavior</t>
         </is>
       </c>
     </row>
@@ -550,7 +550,7 @@
       </c>
       <c r="C4" s="3" t="inlineStr">
         <is>
-          <t>Free Plan Details (Forever Free Tiers)</t>
+          <t>Free Plan Details (Forever Free Tiers / Limits)</t>
         </is>
       </c>
       <c r="D4" s="3" t="inlineStr">
@@ -567,7 +567,7 @@
     <row r="5">
       <c r="A5" s="4" t="inlineStr">
         <is>
-          <t>Sales &amp; CRM</t>
+          <t>Sales</t>
         </is>
       </c>
       <c r="B5" s="5" t="inlineStr">
@@ -577,24 +577,24 @@
       </c>
       <c r="C5" s="6" t="inlineStr">
         <is>
-          <t>Free for up to 3 users. Includes basic Leads, Accounts, Contacts, Deals, tasks, and basic reporting. (10 MB storage cap).</t>
+          <t>Free for up to 3 users. Basic Leads, Accounts, Contacts, Deals, Tasks, and standard reports (10 MB storage cap).</t>
         </is>
       </c>
       <c r="D5" s="6" t="inlineStr">
         <is>
-          <t>Standard / Professional / Enterprise / Ultimate. Unlocks custom fields/modules, sales forecasting, Zia AI, process blueprints, multi-currency, and higher API limits.</t>
+          <t>Standard / Professional / Enterprise / Ultimate. Unlocks custom fields/modules, sales forecasting, Zia AI, process Blueprints, multi-currency, and higher API limits.</t>
         </is>
       </c>
       <c r="E5" s="6" t="inlineStr">
         <is>
-          <t>Account automatically downgrades to Free tier (if &lt;=3 users). Custom fields/modules beyond free limits become read-only/hidden; automated workflows stop running.</t>
+          <t>Automatically downgrades to Free tier (if &lt;=3 users). Custom fields/modules beyond free limits become read-only/hidden; automated workflows stop running.</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="7" t="inlineStr">
         <is>
-          <t>Sales &amp; CRM</t>
+          <t>Sales</t>
         </is>
       </c>
       <c r="B6" s="8" t="inlineStr">
@@ -621,7 +621,7 @@
     <row r="7">
       <c r="A7" s="4" t="inlineStr">
         <is>
-          <t>Sales &amp; CRM</t>
+          <t>Sales</t>
         </is>
       </c>
       <c r="B7" s="5" t="inlineStr">
@@ -631,7 +631,7 @@
       </c>
       <c r="C7" s="6" t="inlineStr">
         <is>
-          <t>Free for 3 users. Includes basic live chat widget, track up to 1,000 site visitors/mo, 100 chat sessions/mo.</t>
+          <t>Free for 3 users. Basic live chat widget, track up to 1,000 site visitors/mo, 100 chat sessions/mo.</t>
         </is>
       </c>
       <c r="D7" s="6" t="inlineStr">
@@ -648,7 +648,7 @@
     <row r="8">
       <c r="A8" s="7" t="inlineStr">
         <is>
-          <t>Sales &amp; CRM</t>
+          <t>Sales</t>
         </is>
       </c>
       <c r="B8" s="8" t="inlineStr">
@@ -675,54 +675,54 @@
     <row r="9">
       <c r="A9" s="4" t="inlineStr">
         <is>
-          <t>Marketing</t>
+          <t>Sales</t>
         </is>
       </c>
       <c r="B9" s="5" t="inlineStr">
         <is>
-          <t>Zoho Campaigns</t>
+          <t>Zoho RouteIQ</t>
         </is>
       </c>
       <c r="C9" s="6" t="inlineStr">
         <is>
-          <t>Free for up to 2,000 contacts. Send up to 6,000 emails/month to your subscriber list. Includes basic templates.</t>
+          <t>15-day Free Trial only.</t>
         </is>
       </c>
       <c r="D9" s="6" t="inlineStr">
         <is>
-          <t>Standard / Professional. Based on subscriber volume. Unlocks automated email workflows/drips, A/B testing, dynamic content, and advanced deliverability tools.</t>
+          <t>Standard / Professional. Visual map routing, sales territory management, and route optimization integrated with CRM.</t>
         </is>
       </c>
       <c r="E9" s="6" t="inlineStr">
         <is>
-          <t>Automatically reverts to 2,000 contact limit. Scheduled automated campaigns/drips freeze; excess contacts remain stored but cannot be emailed.</t>
+          <t>Trial ends and route optimization features lock. Saved route history remains stored in CRM.</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="7" t="inlineStr">
         <is>
-          <t>Marketing</t>
+          <t>Sales</t>
         </is>
       </c>
       <c r="B10" s="8" t="inlineStr">
         <is>
-          <t>Zoho Social</t>
+          <t>Zoho CRM Flex</t>
         </is>
       </c>
       <c r="C10" s="9" t="inlineStr">
         <is>
-          <t>Free for 1 brand. 1 team member, publish to 7 main social networks, basic scheduling.</t>
+          <t>15-day Free Trial only.</t>
         </is>
       </c>
       <c r="D10" s="9" t="inlineStr">
         <is>
-          <t>Standard / Professional / Premium. Adds monitoring dashboards, bulk scheduler, custom roles, social listening, depth reports, and team approvals.</t>
+          <t>Custom developer edition and enterprise composition framework for tailored CRM deployments.</t>
         </is>
       </c>
       <c r="E10" s="9" t="inlineStr">
         <is>
-          <t>Reverts to basic Free tier. Scheduled future posts in queue beyond free limits pause; approval workflows disable.</t>
+          <t>Custom developer limits freeze; production sandbox access turns read-only.</t>
         </is>
       </c>
     </row>
@@ -734,22 +734,22 @@
       </c>
       <c r="B11" s="5" t="inlineStr">
         <is>
-          <t>Zoho Forms</t>
+          <t>Zoho Campaigns</t>
         </is>
       </c>
       <c r="C11" s="6" t="inlineStr">
         <is>
-          <t>Free for 1 user. 3 forms, 500 submissions/month, 200 MB storage, basic field types.</t>
+          <t>Free for up to 2,000 contacts. Send up to 6,000 emails/month to subscriber list. Basic templates.</t>
         </is>
       </c>
       <c r="D11" s="6" t="inlineStr">
         <is>
-          <t>Basic / Standard / Professional / Premium. Unlocks unlimited forms, higher submission volumes, payment integration, PDF generation, and field rules.</t>
+          <t>Standard / Professional (based on subscriber volume). Unlocks automated email workflows/drips, A/B testing, dynamic content, and deliverability tools.</t>
         </is>
       </c>
       <c r="E11" s="6" t="inlineStr">
         <is>
-          <t>Account reverts to 3-form limit. Extra forms are set to inactive (hidden from public view); existing submission data is retained.</t>
+          <t>Reverts to 2,000 contact limit. Scheduled automated campaigns/drips freeze; excess contacts remain stored but cannot be emailed.</t>
         </is>
       </c>
     </row>
@@ -761,22 +761,22 @@
       </c>
       <c r="B12" s="8" t="inlineStr">
         <is>
-          <t>Zoho Survey</t>
+          <t>Zoho Social</t>
         </is>
       </c>
       <c r="C12" s="9" t="inlineStr">
         <is>
-          <t>Free Plan. Unlimited surveys, max 10 questions per survey, 100 responses per survey.</t>
+          <t>Free for 1 brand. 1 team member, publish to 7 main social networks, basic scheduling.</t>
         </is>
       </c>
       <c r="D12" s="9" t="inlineStr">
         <is>
-          <t>Standard / Professional / Enterprise. Unlocks unlimited questions, unlimited responses, skip logic, custom branding, export to PDF/Excel, and multilingual surveys.</t>
+          <t>Standard / Professional / Premium. Adds monitoring dashboards, bulk scheduler, custom roles, social listening, depth reports, and team approvals.</t>
         </is>
       </c>
       <c r="E12" s="9" t="inlineStr">
         <is>
-          <t>Reverts to Free. Surveys exceeding 10 questions block new responses until trimmed; export features lock.</t>
+          <t>Reverts to basic Free tier. Scheduled future posts in queue beyond free limits pause; approval workflows disable.</t>
         </is>
       </c>
     </row>
@@ -788,22 +788,22 @@
       </c>
       <c r="B13" s="5" t="inlineStr">
         <is>
-          <t>Zoho PageSense</t>
+          <t>Zoho Forms</t>
         </is>
       </c>
       <c r="C13" s="6" t="inlineStr">
         <is>
-          <t>15-day Free Trial only. (No perpetual free tier).</t>
+          <t>Free for 1 user. 3 forms, 500 submissions/month, 200 MB storage, basic field types.</t>
         </is>
       </c>
       <c r="D13" s="6" t="inlineStr">
         <is>
-          <t>Standard / Professional / Enterprise. Priced by monthly tracked visitors. Includes Heatmaps, A/B Testing, Form Analytics, Session Recordings.</t>
+          <t>Basic / Standard / Professional / Premium. Unlocks unlimited forms, higher submission volumes, payment integration, PDF generation, and field rules.</t>
         </is>
       </c>
       <c r="E13" s="6" t="inlineStr">
         <is>
-          <t>Trial ends and tracking snippet stops recording visitor sessions. Analytical reports generated during trial remain viewable for a grace period before account locks.</t>
+          <t>Reverts to 3-form limit. Extra forms become set to inactive (hidden from public view); existing submission data is retained.</t>
         </is>
       </c>
     </row>
@@ -815,22 +815,22 @@
       </c>
       <c r="B14" s="8" t="inlineStr">
         <is>
-          <t>Zoho Sites</t>
+          <t>Zoho Survey</t>
         </is>
       </c>
       <c r="C14" s="9" t="inlineStr">
         <is>
-          <t>Free Plan. 1 site, up to 5 pages, top-banner Zoho branding, basic visual builder.</t>
+          <t>Free Plan. Unlimited surveys, max 10 questions per survey, 100 responses per survey.</t>
         </is>
       </c>
       <c r="D14" s="9" t="inlineStr">
         <is>
-          <t>Starter / Pro. Adds unlimited pages, custom domain mapping, removal of Zoho branding, SEO tools, and blog capabilities.</t>
+          <t>Standard / Professional / Enterprise. Unlocks unlimited questions, unlimited responses, skip logic, custom branding, export to PDF/Excel, and multilingual surveys.</t>
         </is>
       </c>
       <c r="E14" s="9" t="inlineStr">
         <is>
-          <t>Downgrades to 5-page limits. Custom domain unbinds (reverts to Zoho subdomain); extra pages become unpublished draft states.</t>
+          <t>Reverts to Free. Surveys exceeding 10 questions block new responses until trimmed; export features lock.</t>
         </is>
       </c>
     </row>
@@ -842,616 +842,1372 @@
       </c>
       <c r="B15" s="5" t="inlineStr">
         <is>
-          <t>Zoho Backstage</t>
+          <t>Zoho PageSense</t>
         </is>
       </c>
       <c r="C15" s="6" t="inlineStr">
         <is>
-          <t>Free Plan. Unlimited free events, basic event portal, ticketing for non-paid tickets.</t>
+          <t>15-day Free Trial only. (No perpetual free tier).</t>
         </is>
       </c>
       <c r="D15" s="6" t="inlineStr">
         <is>
-          <t>Essential / Premium / Ultimate. Unlocks paid ticket sales, sponsor portals, multi-track agendas, badge printing, and event mobile apps.</t>
+          <t>Standard / Professional / Enterprise (priced by monthly tracked visitors). Includes Heatmaps, A/B Testing, Form Analytics, Session Recordings.</t>
         </is>
       </c>
       <c r="E15" s="6" t="inlineStr">
         <is>
-          <t>Reverts to basic free event tier. Paid ticket payment processing disconnects.</t>
+          <t>Trial ends and tracking snippet stops recording visitor sessions. Analytical reports generated during trial remain viewable for a grace period before account locks.</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="7" t="inlineStr">
         <is>
-          <t>Finance &amp; Operations</t>
+          <t>Marketing</t>
         </is>
       </c>
       <c r="B16" s="8" t="inlineStr">
         <is>
-          <t>Zoho Books</t>
+          <t>Zoho Sites</t>
         </is>
       </c>
       <c r="C16" s="9" t="inlineStr">
         <is>
-          <t>Free for small businesses (&lt;$50K annual revenue). 1 user + 1 accountant, manage invoices, expense tracking, track online payments.</t>
+          <t>Free Plan. 1 site, up to 5 pages, top-banner Zoho branding, basic visual builder.</t>
         </is>
       </c>
       <c r="D16" s="9" t="inlineStr">
         <is>
-          <t>Standard / Professional / Premium / Enterprise. Multi-currency, inventory tracking, purchase orders, automated workflows, recurring billing, custom roles.</t>
+          <t>Starter / Pro. Adds unlimited pages, custom domain mapping, removal of Zoho branding, SEO tools, and blog capabilities.</t>
         </is>
       </c>
       <c r="E16" s="9" t="inlineStr">
         <is>
-          <t>Reverts to read-only or restricted state if user count or revenue thresholds are exceeded. Premium features (like custom modules/Blueprints) freeze.</t>
+          <t>Downgrades to 5-page limits. Custom domain unbinds (reverts to Zoho subdomain); extra pages become unpublished draft states.</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="4" t="inlineStr">
         <is>
-          <t>Finance &amp; Operations</t>
+          <t>Marketing</t>
         </is>
       </c>
       <c r="B17" s="5" t="inlineStr">
         <is>
-          <t>Zoho Invoice</t>
+          <t>Zoho Backstage</t>
         </is>
       </c>
       <c r="C17" s="6" t="inlineStr">
         <is>
-          <t>100% Free Forever. Fully featured invoicing, time tracking, portal, payment processing integration. (No paid tiers).</t>
+          <t>Free Plan. Unlimited free events, basic event portal, ticketing for non-paid tickets.</t>
         </is>
       </c>
       <c r="D17" s="6" t="inlineStr">
         <is>
-          <t>N/A (Completely Free). Zoho offers this entirely free as an entry point for freelancers and small businesses.</t>
+          <t>Essential / Premium / Ultimate. Unlocks paid ticket sales, sponsor portals, multi-track agendas, badge printing, and event mobile apps.</t>
         </is>
       </c>
       <c r="E17" s="6" t="inlineStr">
         <is>
-          <t>N/A - No trial expiration or feature locks.</t>
+          <t>Reverts to basic free event tier. Paid ticket payment processing disconnects.</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="7" t="inlineStr">
         <is>
-          <t>Finance &amp; Operations</t>
+          <t>Marketing</t>
         </is>
       </c>
       <c r="B18" s="8" t="inlineStr">
         <is>
-          <t>Zoho Expense</t>
+          <t>Zoho Commerce</t>
         </is>
       </c>
       <c r="C18" s="9" t="inlineStr">
         <is>
-          <t>Free for up to 3 users. Basic expense recording, receipt auto-scan (20 receipts/mo), submit approval flows.</t>
+          <t>15-day Free Trial only.</t>
         </is>
       </c>
       <c r="D18" s="9" t="inlineStr">
         <is>
-          <t>Standard / Premium / Enterprise. Unlocks corporate card feeds, multi-level approvals, policy enforcement, travel requests, and mileage tracking.</t>
+          <t>Starter / Professional / Advanced. Complete e-commerce store builder, inventory sync, order fulfillment, and payment gateways.</t>
         </is>
       </c>
       <c r="E18" s="9" t="inlineStr">
         <is>
-          <t>Downgrades to 3-user free plan. Custom expense policies and automated approval chains default to basic single-step approvals.</t>
+          <t>Storefront becomes inactive after trial ends until a subscription is activated.</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" s="4" t="inlineStr">
         <is>
-          <t>Finance &amp; Operations</t>
+          <t>Marketing</t>
         </is>
       </c>
       <c r="B19" s="5" t="inlineStr">
         <is>
-          <t>Zoho Inventory</t>
+          <t>Zoho Marketing Automation</t>
         </is>
       </c>
       <c r="C19" s="6" t="inlineStr">
         <is>
-          <t>Free Plan. 50 orders/month, 50 shipping labels/month, 1 warehouse, 2 users.</t>
+          <t>15-day Free Trial only.</t>
         </is>
       </c>
       <c r="D19" s="6" t="inlineStr">
         <is>
-          <t>Standard / Professional / Premium / Enterprise. Multi-warehouse management, serial/batch tracking, Shopify/Amazon integrations, high order volumes.</t>
+          <t>Standard / Professional. Multi-channel marketing automation, lead scoring, website tracking, and automated lead nurturing.</t>
         </is>
       </c>
       <c r="E19" s="6" t="inlineStr">
         <is>
-          <t>Reverts to 50 orders/mo limit. When the limit is reached in a month, new order creation blocks until the next billing cycle or upgrade.</t>
+          <t>Automated multi-channel customer journeys freeze; lead scores stop updating.</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" s="7" t="inlineStr">
         <is>
-          <t>Finance &amp; Operations</t>
+          <t>Marketing</t>
         </is>
       </c>
       <c r="B20" s="8" t="inlineStr">
         <is>
-          <t>Zoho Billing (Checkout/Subscriptions)</t>
+          <t>Zoho Publish</t>
         </is>
       </c>
       <c r="C20" s="9" t="inlineStr">
         <is>
-          <t>Free Plan. Max $1,000 monthly revenue limit, 1 user, basic recurring billing &amp; hosted pages.</t>
+          <t>15-day Free Trial only.</t>
         </is>
       </c>
       <c r="D20" s="9" t="inlineStr">
         <is>
-          <t>Standard / Premium / Enterprise. Unlocks usage-based billing, multi-currency, dunning management, advance revenue recognition, higher revenue caps.</t>
+          <t>Local business listing management, review monitoring, and local SEO citations.</t>
         </is>
       </c>
       <c r="E20" s="9" t="inlineStr">
         <is>
-          <t>Upgrading required upon crossing monthly revenue cap. Account enters billing hold (cannot process new recurring cards) until upgraded.</t>
+          <t>Listing sync pauses; location reviews remain viewable in read-only state.</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" s="4" t="inlineStr">
         <is>
-          <t>Finance &amp; Operations</t>
+          <t>Service &amp; Support</t>
         </is>
       </c>
       <c r="B21" s="5" t="inlineStr">
         <is>
-          <t>Zoho Sign</t>
+          <t>Zoho Desk</t>
         </is>
       </c>
       <c r="C21" s="6" t="inlineStr">
         <is>
-          <t>Free for 1 user. 5 digital signatures per month, basic document sign workflow.</t>
+          <t>Free for up to 3 agents. Email ticketing, customer portal, knowledge base, macro actions.</t>
         </is>
       </c>
       <c r="D21" s="6" t="inlineStr">
         <is>
-          <t>Standard / Professional / Enterprise. Unlocks in-bulk send, custom branding, API access, template sharing, signer authentication.</t>
+          <t>Standard / Professional / Enterprise. Unlocks multi-channel tickets (Phone, Social, WhatsApp), SLA agreements, Zia AI support, and agent collision avoidance.</t>
         </is>
       </c>
       <c r="E21" s="6" t="inlineStr">
         <is>
-          <t>Reverts to 5 signatures/mo limit. Unsent signature templates beyond free allowances freeze.</t>
+          <t>Reverts to 3 agents. Tickets from social media/phone integrations stop routing into helpdesk; custom SLAs deactivate.</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" s="7" t="inlineStr">
         <is>
-          <t>HR &amp; Recruitment</t>
+          <t>Service &amp; Support</t>
         </is>
       </c>
       <c r="B22" s="8" t="inlineStr">
         <is>
-          <t>Zoho People</t>
+          <t>Zoho Assist</t>
         </is>
       </c>
       <c r="C22" s="9" t="inlineStr">
         <is>
-          <t>Free for up to 5 users. Employee database, basic time-off management, document storage.</t>
+          <t>Free Plan. 1 remote support technician, 5 unattended remote PCs, basic screen sharing.</t>
         </is>
       </c>
       <c r="D22" s="9" t="inlineStr">
         <is>
-          <t>Essential / Professional / Premium / Enterprise. Adds attendance tracking, shift scheduling, performance management, custom HR workflows, and LMS.</t>
+          <t>Standard / Professional / Enterprise. Adds session recording, file transfer, mobile device support, multi-monitor navigation, and team management.</t>
         </is>
       </c>
       <c r="E22" s="9" t="inlineStr">
         <is>
-          <t>Reverts to 5 employees. Performance reviews, custom HR blueprints, and automated attendance logs pause.</t>
+          <t>Downgrades to 5 unattended computers. Additional configured remote devices disconnect from portal dashboard.</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" s="4" t="inlineStr">
         <is>
-          <t>HR &amp; Recruitment</t>
+          <t>Service &amp; Support</t>
         </is>
       </c>
       <c r="B23" s="5" t="inlineStr">
         <is>
-          <t>Zoho Recruit</t>
+          <t>Zoho Lens</t>
         </is>
       </c>
       <c r="C23" s="6" t="inlineStr">
         <is>
-          <t>Free for 1 recruiter. 1 active job opening, candidate management, basic resume parser.</t>
+          <t>14-day Free Trial only.</t>
         </is>
       </c>
       <c r="D23" s="6" t="inlineStr">
         <is>
-          <t>Standard / Professional / Enterprise. Unlocks unlimited active jobs, job board postings (LinkedIn/Indeed), candidate portals, and offer letter workflows.</t>
+          <t>Standard / Professional. Augmented reality (AR) remote assistance, live video stream annotations, and spatial drawing.</t>
         </is>
       </c>
       <c r="E23" s="6" t="inlineStr">
         <is>
-          <t>Reverts to 1 active job slot. Excess active job posts are automatically unpublished and changed to archived status.</t>
+          <t>AR video sessions lock after trial.</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" s="7" t="inlineStr">
         <is>
-          <t>HR &amp; Recruitment</t>
+          <t>Service &amp; Support</t>
         </is>
       </c>
       <c r="B24" s="8" t="inlineStr">
         <is>
-          <t>Zoho Shifts</t>
+          <t>Zoho FSM</t>
         </is>
       </c>
       <c r="C24" s="9" t="inlineStr">
         <is>
-          <t>Free for up to 7 employees. Basic shift planning, time tracking, employee mobile app.</t>
+          <t>15-day Free Trial only.</t>
         </is>
       </c>
       <c r="D24" s="9" t="inlineStr">
         <is>
-          <t>Standard / Premium. Adds shift swapping, schedule templates, break management, and time-off request policies.</t>
+          <t>Standard / Professional / Enterprise. Field service dispatching, work order management, asset tracking, and field agent mobile apps.</t>
         </is>
       </c>
       <c r="E24" s="9" t="inlineStr">
         <is>
-          <t>Downgrades to basic 7-user schedule viewer. Advanced rules (overtime alerts, swap approvals) stop enforcing.</t>
+          <t>Account switches to read-only mode after trial expires.</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" s="4" t="inlineStr">
         <is>
-          <t>IT, Analytics &amp; Dev</t>
+          <t>Finance &amp; Accounting</t>
         </is>
       </c>
       <c r="B25" s="5" t="inlineStr">
         <is>
-          <t>Zoho Creator</t>
+          <t>Zoho Books</t>
         </is>
       </c>
       <c r="C25" s="6" t="inlineStr">
         <is>
-          <t>Free Plan. 1 custom app, 1 user, 250 MB storage, 1,000 records total.</t>
+          <t>Free for small businesses (&lt;$50K annual revenue). 1 user + 1 accountant, manage invoices, expense tracking, track online payments.</t>
         </is>
       </c>
       <c r="D25" s="6" t="inlineStr">
         <is>
-          <t>Standard / Professional / Enterprise. Build unlimited low-code apps, advanced Deluge script logic, higher storage, multi-user access, REST APIs.</t>
+          <t>Standard / Professional / Premium / Enterprise. Multi-currency, inventory tracking, purchase orders, automated workflows, recurring billing, custom roles.</t>
         </is>
       </c>
       <c r="E25" s="6" t="inlineStr">
         <is>
-          <t>Trial ends/downgrades to 1-app limit. Secondary created apps become disabled/read-only. Executable scripts with high API volume pause.</t>
+          <t>Reverts to read-only or restricted state if user count or revenue thresholds are exceeded. Premium features (like custom modules/Blueprints) freeze.</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" s="7" t="inlineStr">
         <is>
-          <t>IT, Analytics &amp; Dev</t>
+          <t>Finance &amp; Accounting</t>
         </is>
       </c>
       <c r="B26" s="8" t="inlineStr">
         <is>
-          <t>Zoho Analytics</t>
+          <t>Zoho Invoice</t>
         </is>
       </c>
       <c r="C26" s="9" t="inlineStr">
         <is>
-          <t>Free Plan. 2 users, 10,000 rows of data, 5 workspaces, basic reports/dashboards.</t>
+          <t>100% Free Forever. Fully featured invoicing, time tracking, portal, payment processing integration. (No paid tiers).</t>
         </is>
       </c>
       <c r="D26" s="9" t="inlineStr">
         <is>
-          <t>Basic / Standard / Premium / Enterprise. Millions of data rows, automated data connectors, SQL querying, custom alerts, Zia AI insights, and white-labeling.</t>
+          <t>N/A (Completely Free). Zoho offers this entirely free as an entry point for freelancers and small businesses.</t>
         </is>
       </c>
       <c r="E26" s="9" t="inlineStr">
         <is>
-          <t>Downgrades to 10,000 row cap. Automated data syncs from external databases fail/pause if dataset size exceeds free caps.</t>
+          <t>N/A - No trial expiration or feature locks.</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" s="4" t="inlineStr">
         <is>
-          <t>IT, Analytics &amp; Dev</t>
+          <t>Finance &amp; Accounting</t>
         </is>
       </c>
       <c r="B27" s="5" t="inlineStr">
         <is>
-          <t>Zoho Desk</t>
+          <t>Zoho Expense</t>
         </is>
       </c>
       <c r="C27" s="6" t="inlineStr">
         <is>
-          <t>Free for up to 3 agents. Email ticketing, customer portal, knowledge base, macro actions.</t>
+          <t>Free for up to 3 users. Basic expense recording, receipt auto-scan (20 receipts/mo), submit approval flows.</t>
         </is>
       </c>
       <c r="D27" s="6" t="inlineStr">
         <is>
-          <t>Standard / Professional / Enterprise. Unlocks multi-channel tickets (Phone, Social, WhatsApp), SLA agreements, Zia AI support, and agent collision avoidance.</t>
+          <t>Standard / Premium / Enterprise. Unlocks corporate card feeds, multi-level approvals, policy enforcement, travel requests, and mileage tracking.</t>
         </is>
       </c>
       <c r="E27" s="6" t="inlineStr">
         <is>
-          <t>Reverts to 3 agents. Tickets from social media/phone integrations stop routing into the helpdesk system; custom SLAs deactivate.</t>
+          <t>Downgrades to 3-user free plan. Custom expense policies and automated approval chains default to basic single-step approvals.</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" s="7" t="inlineStr">
         <is>
-          <t>IT, Analytics &amp; Dev</t>
+          <t>Finance &amp; Accounting</t>
         </is>
       </c>
       <c r="B28" s="8" t="inlineStr">
         <is>
-          <t>Zoho Assist</t>
+          <t>Zoho Inventory</t>
         </is>
       </c>
       <c r="C28" s="9" t="inlineStr">
         <is>
-          <t>Free Plan. 1 remote support technician, 5 unattended remote PCs, basic screen sharing.</t>
+          <t>Free Plan. 50 orders/month, 50 shipping labels/month, 1 warehouse, 2 users.</t>
         </is>
       </c>
       <c r="D28" s="9" t="inlineStr">
         <is>
-          <t>Standard / Professional / Enterprise. Adds session recording, file transfer, mobile device support, multi-monitor navigation, and team management.</t>
+          <t>Standard / Professional / Premium / Enterprise. Multi-warehouse management, serial/batch tracking, Shopify/Amazon integrations, high order volumes.</t>
         </is>
       </c>
       <c r="E28" s="9" t="inlineStr">
         <is>
-          <t>Downgrades to 5 unattended computers. Additional configured remote devices disconnect from the portal dashboard.</t>
+          <t>Reverts to 50 orders/mo limit. When limit is reached in a month, new order creation blocks until next billing cycle or upgrade.</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" s="4" t="inlineStr">
         <is>
-          <t>IT, Analytics &amp; Dev</t>
+          <t>Finance &amp; Accounting</t>
         </is>
       </c>
       <c r="B29" s="5" t="inlineStr">
         <is>
-          <t>Zoho Vault</t>
+          <t>Zoho Billing</t>
         </is>
       </c>
       <c r="C29" s="6" t="inlineStr">
         <is>
-          <t>Free Forever for Personal Use. Unlimited passwords, secure cloud storage, multi-device sync.</t>
+          <t>Free Plan. Max $1,000 monthly revenue limit, 1 user, basic recurring billing &amp; hosted pages.</t>
         </is>
       </c>
       <c r="D29" s="6" t="inlineStr">
         <is>
-          <t>Standard / Professional / Enterprise. Unlocks team password sharing, role-based access, password assessment, user provisioning, and active directory sync.</t>
+          <t>Standard / Premium / Enterprise. Unlocks usage-based billing, multi-currency, dunning management, advance revenue recognition, higher revenue caps.</t>
         </is>
       </c>
       <c r="E29" s="6" t="inlineStr">
         <is>
-          <t>For business trials: Reverts to individual vault mode. Shared team password folders locked for non-owners.</t>
+          <t>Upgrading required upon crossing monthly revenue cap. Account enters billing hold (cannot process new recurring cards) until upgraded.</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" s="7" t="inlineStr">
         <is>
-          <t>IT, Analytics &amp; Dev</t>
+          <t>Finance &amp; Accounting</t>
         </is>
       </c>
       <c r="B30" s="8" t="inlineStr">
         <is>
-          <t>Zoho Site24x7</t>
+          <t>Zoho Checkout</t>
         </is>
       </c>
       <c r="C30" s="9" t="inlineStr">
         <is>
-          <t>Free Plan. Monitor up to 5 websites/servers at 10-minute check intervals.</t>
+          <t>Free Plan. Up to 50 payments, 1 user.</t>
         </is>
       </c>
       <c r="D30" s="9" t="inlineStr">
         <is>
-          <t>Pro / Enterprise. 1-minute check intervals, synthetic transaction monitoring, APM, network monitoring, SMS alerts.</t>
+          <t>Standard / Professional. Custom payment pages, recurring payments, multi-currency, and transaction confirmations.</t>
         </is>
       </c>
       <c r="E30" s="9" t="inlineStr">
         <is>
-          <t>Downgrades to 5 basic monitors. Advanced APM agents stop sending metrics; alert frequency drops to 10-min intervals.</t>
+          <t>Reverts to 50 payment cap; payment forms deactivate when limit is exceeded.</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" s="4" t="inlineStr">
         <is>
-          <t>Office &amp; Collaboration</t>
+          <t>Finance &amp; Accounting</t>
         </is>
       </c>
       <c r="B31" s="5" t="inlineStr">
         <is>
-          <t>Zoho Mail</t>
+          <t>Zoho Payroll</t>
         </is>
       </c>
       <c r="C31" s="6" t="inlineStr">
         <is>
-          <t>Free for up to 5 users. 5 GB storage/user, web/mobile app access only (NO IMAP/POP3).</t>
+          <t>Free for up to 10 employees (In specific jurisdictions/regions).</t>
         </is>
       </c>
       <c r="D31" s="6" t="inlineStr">
         <is>
-          <t>Mail Lite / Mail Premium / Workplace. Adds IMAP/POP/ActiveSync (Outlook/Apple Mail support), custom routing, 10 GB to 50+ GB storage/user, domain aliases.</t>
+          <t>Standard Plan. Automated tax calculation, direct deposit, compliance management, and payslip generation.</t>
         </is>
       </c>
       <c r="E31" s="6" t="inlineStr">
         <is>
-          <t>Downgrades to webmail-only access. External email clients (Outlook/Thunderbird) lose connection via IMAP/POP.</t>
+          <t>Payroll runs freeze if employee limits exceed free threshold.</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" s="7" t="inlineStr">
         <is>
-          <t>Office &amp; Collaboration</t>
+          <t>Finance &amp; Accounting</t>
         </is>
       </c>
       <c r="B32" s="8" t="inlineStr">
         <is>
-          <t>Zoho WorkDrive</t>
+          <t>Zoho Practice</t>
         </is>
       </c>
       <c r="C32" s="9" t="inlineStr">
         <is>
-          <t>15-day Free Trial only. (15 days full Enterprise features; no perpetual free plan for teams).</t>
+          <t>Free for accounting firms.</t>
         </is>
       </c>
       <c r="D32" s="9" t="inlineStr">
         <is>
-          <t>Starter / Team / Business. Scalable cloud storage (1 TB+ per team), granular file permissions, Admin console, Zoho Office suite integration.</t>
+          <t>Pro Tiers. Client management portal, task tracking, document sharing, and client accounting integration.</t>
         </is>
       </c>
       <c r="E32" s="9" t="inlineStr">
         <is>
-          <t>Account becomes read-only. Users can view/download files created during trial, but uploading new files or editing online is blocked until a plan is chosen.</t>
+          <t>Advanced firm management workflows pause; client document access remains open.</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" s="4" t="inlineStr">
         <is>
-          <t>Office &amp; Collaboration</t>
+          <t>Human Resources</t>
         </is>
       </c>
       <c r="B33" s="5" t="inlineStr">
         <is>
-          <t>Zoho Cliq</t>
+          <t>Zoho People</t>
         </is>
       </c>
       <c r="C33" s="6" t="inlineStr">
         <is>
-          <t>Free Plan. 10,000 searchable messages, 100 GB storage for org, up to 100 participants/channel.</t>
+          <t>Free for up to 5 users. Employee database, basic time-off management, document storage.</t>
         </is>
       </c>
       <c r="D33" s="6" t="inlineStr">
         <is>
-          <t>Unlimited Plan. Unlimited message search history, custom bots, screen sharing, read receipts, custom domain, and guest access.</t>
+          <t>Essential / Professional / Premium / Enterprise. Adds attendance tracking, shift scheduling, performance management, custom HR workflows, and LMS.</t>
         </is>
       </c>
       <c r="E33" s="6" t="inlineStr">
         <is>
-          <t>Downgrades to Free. Message history beyond the most recent 10,000 messages is hidden from search results (restored upon upgrade).</t>
+          <t>Reverts to 5 employees. Performance reviews, custom HR blueprints, and automated attendance logs pause.</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" s="7" t="inlineStr">
         <is>
-          <t>Office &amp; Collaboration</t>
+          <t>Human Resources</t>
         </is>
       </c>
       <c r="B34" s="8" t="inlineStr">
         <is>
-          <t>Zoho Projects</t>
+          <t>Zoho Recruit</t>
         </is>
       </c>
       <c r="C34" s="9" t="inlineStr">
         <is>
-          <t>Free for up to 3 users. 2 active projects, 5 GB storage, Gantt charts, basic task management.</t>
+          <t>Free for 1 recruiter. 1 active job opening, candidate management, basic resume parser.</t>
         </is>
       </c>
       <c r="D34" s="9" t="inlineStr">
         <is>
-          <t>Premium / Enterprise. Unlimited projects, subtasks, custom task statuses, task blueprints, time logging, expense tracking, and resource utilization.</t>
+          <t>Standard / Professional / Enterprise. Unlocks unlimited active jobs, job board postings (LinkedIn/Indeed), candidate portals, and offer letter workflows.</t>
         </is>
       </c>
       <c r="E34" s="9" t="inlineStr">
         <is>
-          <t>Downgrades to 2 active projects. Additional projects become archived/read-only; task automation workflows halt.</t>
+          <t>Reverts to 1 active job slot. Excess active job posts are automatically unpublished and changed to archived status.</t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="A35" s="4" t="inlineStr">
         <is>
-          <t>Office &amp; Collaboration</t>
+          <t>Human Resources</t>
         </is>
       </c>
       <c r="B35" s="5" t="inlineStr">
         <is>
-          <t>Zoho Meeting</t>
+          <t>Zoho Shifts</t>
         </is>
       </c>
       <c r="C35" s="6" t="inlineStr">
         <is>
-          <t>Free Plan. Up to 100 meeting participants, 60-minute duration limit, screen sharing.</t>
+          <t>Free for up to 7 employees. Basic shift planning, time tracking, employee mobile app.</t>
         </is>
       </c>
       <c r="D35" s="6" t="inlineStr">
         <is>
-          <t>Meeting / Webinar Plans. 24-hour meeting duration, cloud recording storage, co-hosts, custom branding, and interactive polls.</t>
+          <t>Standard / Premium. Adds shift swapping, schedule templates, break management, and time-off request policies.</t>
         </is>
       </c>
       <c r="E35" s="6" t="inlineStr">
         <is>
-          <t>Reverts to 60-min cap. Cloud recordings saved during trial are retained temporarily but require paid storage for long-term retention.</t>
+          <t>Downgrades to basic 7-user schedule viewer. Advanced rules (overtime alerts, swap approvals) stop enforcing.</t>
         </is>
       </c>
     </row>
     <row r="36">
       <c r="A36" s="7" t="inlineStr">
         <is>
-          <t>Office &amp; Collaboration</t>
+          <t>Human Resources</t>
         </is>
       </c>
       <c r="B36" s="8" t="inlineStr">
         <is>
-          <t>Zoho Writer / Sheet / Show</t>
+          <t>Zoho Workerly</t>
         </is>
       </c>
       <c r="C36" s="9" t="inlineStr">
         <is>
-          <t>100% Free Forever. Complete cloud office productivity suite.</t>
+          <t>Free for 1 recruiter.</t>
         </is>
       </c>
       <c r="D36" s="9" t="inlineStr">
         <is>
-          <t>Included with Zoho WorkDrive / Workplace. High-tier features tied to team storage and administrative controls.</t>
+          <t>Standard / Professional. Specialized temporary staffing platform, temp scheduling, time cards, and client invoicing.</t>
         </is>
       </c>
       <c r="E36" s="9" t="inlineStr">
         <is>
-          <t>N/A - Standard document creation is entirely free for individuals.</t>
+          <t>Downgrades to 1-recruiter limit; active temp assignment dispatching locks.</t>
         </is>
       </c>
     </row>
     <row r="37">
       <c r="A37" s="4" t="inlineStr">
         <is>
-          <t>Office &amp; Collaboration</t>
+          <t>Human Resources</t>
         </is>
       </c>
       <c r="B37" s="5" t="inlineStr">
         <is>
+          <t>Zoho Learn</t>
+        </is>
+      </c>
+      <c r="C37" s="6" t="inlineStr">
+        <is>
+          <t>Free Plan. Up to 5 users, basic knowledge base, 1 course creation.</t>
+        </is>
+      </c>
+      <c r="D37" s="6" t="inlineStr">
+        <is>
+          <t>Express / Professional. Full Learning Management System (LMS), quiz creation, course certification, and custom roles.</t>
+        </is>
+      </c>
+      <c r="E37" s="6" t="inlineStr">
+        <is>
+          <t>Reverts to 5 users and 1 course.</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="7" t="inlineStr">
+        <is>
+          <t>Project &amp; Work Management</t>
+        </is>
+      </c>
+      <c r="B38" s="8" t="inlineStr">
+        <is>
+          <t>Zoho Projects</t>
+        </is>
+      </c>
+      <c r="C38" s="9" t="inlineStr">
+        <is>
+          <t>Free for up to 3 users. Includes 2 active projects, 5 GB storage, Gantt charts, and basic task management.</t>
+        </is>
+      </c>
+      <c r="D38" s="9" t="inlineStr">
+        <is>
+          <t>Premium / Enterprise. Unlocks unlimited projects, subtasks, custom task statuses, task blueprints, issue tracking, time logging, expense tracking, and resource utilization.</t>
+        </is>
+      </c>
+      <c r="E38" s="9" t="inlineStr">
+        <is>
+          <t>Downgrades to 2 active projects. Excess projects become archived/read-only; task automation workflows halt.</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="4" t="inlineStr">
+        <is>
+          <t>Project &amp; Work Management</t>
+        </is>
+      </c>
+      <c r="B39" s="5" t="inlineStr">
+        <is>
+          <t>Zoho Sprints</t>
+        </is>
+      </c>
+      <c r="C39" s="6" t="inlineStr">
+        <is>
+          <t>Free for up to 3 users. Includes 2 active projects, 500 MB storage, basic agile backlogs, and sprint planning.</t>
+        </is>
+      </c>
+      <c r="D39" s="6" t="inlineStr">
+        <is>
+          <t>Standard / Premium. Unlocks unlimited projects &amp; sprints, release management, epic tracking, timesheets, and velocity charts.</t>
+        </is>
+      </c>
+      <c r="E39" s="6" t="inlineStr">
+        <is>
+          <t>Reverts to 2 active projects. Extra projects lock in read-only mode; active sprint automations pause.</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" s="7" t="inlineStr">
+        <is>
+          <t>Project &amp; Work Management</t>
+        </is>
+      </c>
+      <c r="B40" s="8" t="inlineStr">
+        <is>
+          <t>Zoho BugTracker</t>
+        </is>
+      </c>
+      <c r="C40" s="9" t="inlineStr">
+        <is>
+          <t>Free for up to 3 users. Includes 2 projects, bug reporting, and basic issue tracking.</t>
+        </is>
+      </c>
+      <c r="D40" s="9" t="inlineStr">
+        <is>
+          <t>Standard / Premium. Unlocks unlimited projects, custom issue workflows, SLA rules, and time tracking.</t>
+        </is>
+      </c>
+      <c r="E40" s="9" t="inlineStr">
+        <is>
+          <t>Reverts to Free limit of 2 projects. Extra issue tracking repositories freeze.</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" s="4" t="inlineStr">
+        <is>
+          <t>Project &amp; Work Management</t>
+        </is>
+      </c>
+      <c r="B41" s="5" t="inlineStr">
+        <is>
+          <t>Zoho Contracts</t>
+        </is>
+      </c>
+      <c r="C41" s="6" t="inlineStr">
+        <is>
+          <t>15-day Free Trial only.</t>
+        </is>
+      </c>
+      <c r="D41" s="6" t="inlineStr">
+        <is>
+          <t>Standard / Professional. End-to-end contract lifecycle management, authoring, approval workflows, and obligation tracking.</t>
+        </is>
+      </c>
+      <c r="E41" s="6" t="inlineStr">
+        <is>
+          <t>Contracts remain viewable in read-only state; active approval and renewal alerts cease.</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" s="7" t="inlineStr">
+        <is>
+          <t>Office Productivity</t>
+        </is>
+      </c>
+      <c r="B42" s="8" t="inlineStr">
+        <is>
+          <t>Zoho Writer</t>
+        </is>
+      </c>
+      <c r="C42" s="9" t="inlineStr">
+        <is>
+          <t>100% Free Forever for individual word processing.</t>
+        </is>
+      </c>
+      <c r="D42" s="9" t="inlineStr">
+        <is>
+          <t>Included with Workplace/WorkDrive. Real-time collaboration, fillable document templates, mail merge, and electronic signatures.</t>
+        </is>
+      </c>
+      <c r="E42" s="9" t="inlineStr">
+        <is>
+          <t>N/A - Standalone document editor is completely free.</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" s="4" t="inlineStr">
+        <is>
+          <t>Office Productivity</t>
+        </is>
+      </c>
+      <c r="B43" s="5" t="inlineStr">
+        <is>
+          <t>Zoho Sheet</t>
+        </is>
+      </c>
+      <c r="C43" s="6" t="inlineStr">
+        <is>
+          <t>100% Free Forever for individual spreadsheet creation.</t>
+        </is>
+      </c>
+      <c r="D43" s="6" t="inlineStr">
+        <is>
+          <t>Included with Workplace/WorkDrive. Automated data cleaning, custom macros, Zia AI analysis, and external data connectors.</t>
+        </is>
+      </c>
+      <c r="E43" s="6" t="inlineStr">
+        <is>
+          <t>N/A - Standalone spreadsheet editor is completely free.</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" s="7" t="inlineStr">
+        <is>
+          <t>Office Productivity</t>
+        </is>
+      </c>
+      <c r="B44" s="8" t="inlineStr">
+        <is>
+          <t>Zoho Show</t>
+        </is>
+      </c>
+      <c r="C44" s="9" t="inlineStr">
+        <is>
+          <t>100% Free Forever for presentation creation.</t>
+        </is>
+      </c>
+      <c r="D44" s="9" t="inlineStr">
+        <is>
+          <t>Included with Workplace/WorkDrive. Interactive presentation deck builder, smart animation, and broadcasting.</t>
+        </is>
+      </c>
+      <c r="E44" s="9" t="inlineStr">
+        <is>
+          <t>N/A - Standalone presentation editor is completely free.</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" s="4" t="inlineStr">
+        <is>
+          <t>Office Productivity</t>
+        </is>
+      </c>
+      <c r="B45" s="5" t="inlineStr">
+        <is>
           <t>Zoho Notebook</t>
         </is>
       </c>
-      <c r="C37" s="6" t="inlineStr">
-        <is>
-          <t>100% Free Forever. Cross-platform note-taking, card organization, audio notes.</t>
-        </is>
-      </c>
-      <c r="D37" s="6" t="inlineStr">
-        <is>
-          <t>Pro Version available. Adds file attachment size increases, custom covers, and version history.</t>
-        </is>
-      </c>
-      <c r="E37" s="6" t="inlineStr">
-        <is>
-          <t>Basic note-taking and sync remain free forever without data lock.</t>
+      <c r="C45" s="6" t="inlineStr">
+        <is>
+          <t>100% Free Forever cross-platform note app.</t>
+        </is>
+      </c>
+      <c r="D45" s="6" t="inlineStr">
+        <is>
+          <t>Pro Version available. Increases file attachment sizes, custom card covers, and version history.</t>
+        </is>
+      </c>
+      <c r="E45" s="6" t="inlineStr">
+        <is>
+          <t>N/A - Core note taking and cross-device sync remain free.</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" s="7" t="inlineStr">
+        <is>
+          <t>Office Productivity</t>
+        </is>
+      </c>
+      <c r="B46" s="8" t="inlineStr">
+        <is>
+          <t>Zoho WorkDrive</t>
+        </is>
+      </c>
+      <c r="C46" s="9" t="inlineStr">
+        <is>
+          <t>15-day Free Trial only. (No perpetual free plan for team workspaces).</t>
+        </is>
+      </c>
+      <c r="D46" s="9" t="inlineStr">
+        <is>
+          <t>Starter / Team / Business. Scalable cloud storage (1 TB+ per team), granular file permissions, Admin console, Zoho Office suite integration.</t>
+        </is>
+      </c>
+      <c r="E46" s="9" t="inlineStr">
+        <is>
+          <t>Account becomes read-only. Users can view/download files created during trial, but uploading new files or editing online is blocked until a plan is chosen.</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" s="4" t="inlineStr">
+        <is>
+          <t>Office Productivity</t>
+        </is>
+      </c>
+      <c r="B47" s="5" t="inlineStr">
+        <is>
+          <t>Zoho Sign</t>
+        </is>
+      </c>
+      <c r="C47" s="6" t="inlineStr">
+        <is>
+          <t>Free for 1 user. 5 digital signatures per month, basic document sign workflow.</t>
+        </is>
+      </c>
+      <c r="D47" s="6" t="inlineStr">
+        <is>
+          <t>Standard / Professional / Enterprise. Unlocks in-bulk send, custom branding, API access, template sharing, signer authentication.</t>
+        </is>
+      </c>
+      <c r="E47" s="6" t="inlineStr">
+        <is>
+          <t>Reverts to 5 signatures/mo limit. Unsent signature templates beyond free allowances freeze.</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" s="7" t="inlineStr">
+        <is>
+          <t>Office Productivity</t>
+        </is>
+      </c>
+      <c r="B48" s="8" t="inlineStr">
+        <is>
+          <t>Zoho Mail</t>
+        </is>
+      </c>
+      <c r="C48" s="9" t="inlineStr">
+        <is>
+          <t>Free for up to 5 users. 5 GB storage/user, web/mobile app access only (NO IMAP/POP3).</t>
+        </is>
+      </c>
+      <c r="D48" s="9" t="inlineStr">
+        <is>
+          <t>Mail Lite / Mail Premium / Workplace. Adds IMAP/POP/ActiveSync (Outlook/Apple Mail support), custom routing, 10 GB to 50+ GB storage/user, domain aliases.</t>
+        </is>
+      </c>
+      <c r="E48" s="9" t="inlineStr">
+        <is>
+          <t>Downgrades to webmail-only access. External email clients (Outlook/Thunderbird) lose connection via IMAP/POP.</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" s="4" t="inlineStr">
+        <is>
+          <t>Office Productivity</t>
+        </is>
+      </c>
+      <c r="B49" s="5" t="inlineStr">
+        <is>
+          <t>Zoho Cliq</t>
+        </is>
+      </c>
+      <c r="C49" s="6" t="inlineStr">
+        <is>
+          <t>Free Plan. 10,000 searchable messages, 100 GB storage for org, up to 100 participants/channel.</t>
+        </is>
+      </c>
+      <c r="D49" s="6" t="inlineStr">
+        <is>
+          <t>Unlimited Plan. Unlimited message search history, custom bots, screen sharing, read receipts, custom domain, and guest access.</t>
+        </is>
+      </c>
+      <c r="E49" s="6" t="inlineStr">
+        <is>
+          <t>Downgrades to Free. Message history beyond the most recent 10,000 messages is hidden from search results (restored upon upgrade).</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" s="7" t="inlineStr">
+        <is>
+          <t>Office Productivity</t>
+        </is>
+      </c>
+      <c r="B50" s="8" t="inlineStr">
+        <is>
+          <t>Zoho Meeting</t>
+        </is>
+      </c>
+      <c r="C50" s="9" t="inlineStr">
+        <is>
+          <t>Free Plan. Up to 100 meeting participants, 60-minute duration limit, screen sharing.</t>
+        </is>
+      </c>
+      <c r="D50" s="9" t="inlineStr">
+        <is>
+          <t>Meeting / Webinar Plans. 24-hour meeting duration, cloud recording storage, co-hosts, custom branding, and interactive polls.</t>
+        </is>
+      </c>
+      <c r="E50" s="9" t="inlineStr">
+        <is>
+          <t>Reverts to 60-min cap. Cloud recordings saved during trial are retained temporarily but require paid storage for long-term retention.</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" s="4" t="inlineStr">
+        <is>
+          <t>Office Productivity</t>
+        </is>
+      </c>
+      <c r="B51" s="5" t="inlineStr">
+        <is>
+          <t>Zoho Connect</t>
+        </is>
+      </c>
+      <c r="C51" s="6" t="inlineStr">
+        <is>
+          <t>Free Plan. Up to 25 users, basic team feeds, channels, and groups.</t>
+        </is>
+      </c>
+      <c r="D51" s="6" t="inlineStr">
+        <is>
+          <t>Enterprise Plan. Unlocks unlimited users, custom internal intranet pages, polls, user manuals, and external guest access.</t>
+        </is>
+      </c>
+      <c r="E51" s="6" t="inlineStr">
+        <is>
+          <t>Reverts to 25 user limit; custom intranet pages turn read-only.</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" s="7" t="inlineStr">
+        <is>
+          <t>Office Productivity</t>
+        </is>
+      </c>
+      <c r="B52" s="8" t="inlineStr">
+        <is>
+          <t>Zoho Voice</t>
+        </is>
+      </c>
+      <c r="C52" s="9" t="inlineStr">
+        <is>
+          <t>15-day Free Trial only.</t>
+        </is>
+      </c>
+      <c r="D52" s="9" t="inlineStr">
+        <is>
+          <t>Basic / Standard / Contact Center. Cloud PBX, business phone numbers, call queues, and IVR.</t>
+        </is>
+      </c>
+      <c r="E52" s="9" t="inlineStr">
+        <is>
+          <t>Inbound/outbound calling stops when trial or credits expire.</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" s="4" t="inlineStr">
+        <is>
+          <t>Office Productivity</t>
+        </is>
+      </c>
+      <c r="B53" s="5" t="inlineStr">
+        <is>
+          <t>Zoho ToDo</t>
+        </is>
+      </c>
+      <c r="C53" s="6" t="inlineStr">
+        <is>
+          <t>100% Free Forever.</t>
+        </is>
+      </c>
+      <c r="D53" s="6" t="inlineStr">
+        <is>
+          <t>Included with Zoho Mail/Workplace. Basic personal and team task checklist manager.</t>
+        </is>
+      </c>
+      <c r="E53" s="6" t="inlineStr">
+        <is>
+          <t>N/A - Free tool.</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" s="7" t="inlineStr">
+        <is>
+          <t>Office Productivity</t>
+        </is>
+      </c>
+      <c r="B54" s="8" t="inlineStr">
+        <is>
+          <t>Zoho Calendar</t>
+        </is>
+      </c>
+      <c r="C54" s="9" t="inlineStr">
+        <is>
+          <t>100% Free Forever.</t>
+        </is>
+      </c>
+      <c r="D54" s="9" t="inlineStr">
+        <is>
+          <t>Included with Zoho Mail/Workplace. Shared business calendars, resource booking, and event scheduling.</t>
+        </is>
+      </c>
+      <c r="E54" s="9" t="inlineStr">
+        <is>
+          <t>N/A - Free tool.</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" s="4" t="inlineStr">
+        <is>
+          <t>Office Productivity</t>
+        </is>
+      </c>
+      <c r="B55" s="5" t="inlineStr">
+        <is>
+          <t>Zoho Streams</t>
+        </is>
+      </c>
+      <c r="C55" s="6" t="inlineStr">
+        <is>
+          <t>100% Free Forever within Zoho Mail.</t>
+        </is>
+      </c>
+      <c r="D55" s="6" t="inlineStr">
+        <is>
+          <t>Social-style email commenting and discussion feeds built directly inside Zoho Mail.</t>
+        </is>
+      </c>
+      <c r="E55" s="6" t="inlineStr">
+        <is>
+          <t>N/A - Free integration.</t>
+        </is>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" s="7" t="inlineStr">
+        <is>
+          <t>IT &amp; Security</t>
+        </is>
+      </c>
+      <c r="B56" s="8" t="inlineStr">
+        <is>
+          <t>Zoho Creator</t>
+        </is>
+      </c>
+      <c r="C56" s="9" t="inlineStr">
+        <is>
+          <t>Free Plan. 1 custom app, 1 user, 250 MB storage, 1,000 records total.</t>
+        </is>
+      </c>
+      <c r="D56" s="9" t="inlineStr">
+        <is>
+          <t>Standard / Professional / Enterprise. Build unlimited low-code apps, advanced Deluge script logic, higher storage, multi-user access, REST APIs.</t>
+        </is>
+      </c>
+      <c r="E56" s="9" t="inlineStr">
+        <is>
+          <t>Trial ends/downgrades to 1-app limit. Secondary created apps become disabled/read-only. Executable scripts with high API volume pause.</t>
+        </is>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" s="4" t="inlineStr">
+        <is>
+          <t>IT &amp; Security</t>
+        </is>
+      </c>
+      <c r="B57" s="5" t="inlineStr">
+        <is>
+          <t>Zoho Analytics</t>
+        </is>
+      </c>
+      <c r="C57" s="6" t="inlineStr">
+        <is>
+          <t>Free Plan. 2 users, 10,000 rows of data, 5 workspaces, basic reports/dashboards.</t>
+        </is>
+      </c>
+      <c r="D57" s="6" t="inlineStr">
+        <is>
+          <t>Basic / Standard / Premium / Enterprise. Millions of data rows, automated data connectors, SQL querying, custom alerts, Zia AI insights, and white-labeling.</t>
+        </is>
+      </c>
+      <c r="E57" s="6" t="inlineStr">
+        <is>
+          <t>Downgrades to 10,000 row cap. Automated data syncs from external databases fail/pause if dataset size exceeds free caps.</t>
+        </is>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" s="7" t="inlineStr">
+        <is>
+          <t>IT &amp; Security</t>
+        </is>
+      </c>
+      <c r="B58" s="8" t="inlineStr">
+        <is>
+          <t>Zoho Vault</t>
+        </is>
+      </c>
+      <c r="C58" s="9" t="inlineStr">
+        <is>
+          <t>Free Forever for Personal Use. Unlimited passwords, secure cloud storage, multi-device sync.</t>
+        </is>
+      </c>
+      <c r="D58" s="9" t="inlineStr">
+        <is>
+          <t>Standard / Professional / Enterprise. Unlocks team password sharing, role-based access, password assessment, user provisioning, and active directory sync.</t>
+        </is>
+      </c>
+      <c r="E58" s="9" t="inlineStr">
+        <is>
+          <t>For business trials: Reverts to individual vault mode. Shared team password folders locked for non-owners.</t>
+        </is>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" s="4" t="inlineStr">
+        <is>
+          <t>IT &amp; Security</t>
+        </is>
+      </c>
+      <c r="B59" s="5" t="inlineStr">
+        <is>
+          <t>Zoho Site24x7</t>
+        </is>
+      </c>
+      <c r="C59" s="6" t="inlineStr">
+        <is>
+          <t>Free Plan. Monitor up to 5 websites/servers at 10-minute check intervals.</t>
+        </is>
+      </c>
+      <c r="D59" s="6" t="inlineStr">
+        <is>
+          <t>Pro / Enterprise. 1-minute check intervals, synthetic transaction monitoring, APM, network monitoring, SMS alerts.</t>
+        </is>
+      </c>
+      <c r="E59" s="6" t="inlineStr">
+        <is>
+          <t>Downgrades to 5 basic monitors. Advanced APM agents stop sending metrics; alert frequency drops to 10-min intervals.</t>
+        </is>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" s="7" t="inlineStr">
+        <is>
+          <t>IT &amp; Security</t>
+        </is>
+      </c>
+      <c r="B60" s="8" t="inlineStr">
+        <is>
+          <t>Zoho Flow</t>
+        </is>
+      </c>
+      <c r="C60" s="9" t="inlineStr">
+        <is>
+          <t>Free Plan. 100 tasks/month, 5 flows, 15-minute check interval.</t>
+        </is>
+      </c>
+      <c r="D60" s="9" t="inlineStr">
+        <is>
+          <t>Standard / Professional / Enterprise. Thousands of tasks/mo, multi-step webhooks, custom Deluge scripts, and instant triggers.</t>
+        </is>
+      </c>
+      <c r="E60" s="9" t="inlineStr">
+        <is>
+          <t>Reverts to 100 tasks/mo limit. Flows beyond the 5th pause execution.</t>
+        </is>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" s="4" t="inlineStr">
+        <is>
+          <t>IT &amp; Security</t>
+        </is>
+      </c>
+      <c r="B61" s="5" t="inlineStr">
+        <is>
+          <t>Zoho DataPrep</t>
+        </is>
+      </c>
+      <c r="C61" s="6" t="inlineStr">
+        <is>
+          <t>15-day Free Trial only.</t>
+        </is>
+      </c>
+      <c r="D61" s="6" t="inlineStr">
+        <is>
+          <t>Standard / Enterprise. Self-service data preparation, cleaning, transformation, and pipeline automation.</t>
+        </is>
+      </c>
+      <c r="E61" s="6" t="inlineStr">
+        <is>
+          <t>Data pipelines freeze after trial expiration.</t>
+        </is>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" s="7" t="inlineStr">
+        <is>
+          <t>IT &amp; Security</t>
+        </is>
+      </c>
+      <c r="B62" s="8" t="inlineStr">
+        <is>
+          <t>ZeptoMail by Zoho</t>
+        </is>
+      </c>
+      <c r="C62" s="9" t="inlineStr">
+        <is>
+          <t>Free Credits on sign-up (Transactional Email Service).</t>
+        </is>
+      </c>
+      <c r="D62" s="9" t="inlineStr">
+        <is>
+          <t>Pay-as-you-go email credits for application transaction emails (password resets, receipt emails).</t>
+        </is>
+      </c>
+      <c r="E62" s="9" t="inlineStr">
+        <is>
+          <t>Transactional email sending halts when credit balance reaches zero.</t>
+        </is>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" s="4" t="inlineStr">
+        <is>
+          <t>IT &amp; Security</t>
+        </is>
+      </c>
+      <c r="B63" s="5" t="inlineStr">
+        <is>
+          <t>Zoho Catalyst</t>
+        </is>
+      </c>
+      <c r="C63" s="6" t="inlineStr">
+        <is>
+          <t>Free Tier / Generous Monthly Allowance.</t>
+        </is>
+      </c>
+      <c r="D63" s="6" t="inlineStr">
+        <is>
+          <t>Pay-as-you-go serverless developer platform (Functions, DB, Storage, Event Listeners).</t>
+        </is>
+      </c>
+      <c r="E63" s="6" t="inlineStr">
+        <is>
+          <t>Free limits apply monthly; usage beyond cap requires billing profile.</t>
+        </is>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" s="7" t="inlineStr">
+        <is>
+          <t>IT &amp; Security</t>
+        </is>
+      </c>
+      <c r="B64" s="8" t="inlineStr">
+        <is>
+          <t>Zoho Directory</t>
+        </is>
+      </c>
+      <c r="C64" s="9" t="inlineStr">
+        <is>
+          <t>Free for basic identity management.</t>
+        </is>
+      </c>
+      <c r="D64" s="9" t="inlineStr">
+        <is>
+          <t>Standard / Premium. Cloud IAM, single sign-on (SSO), multi-factor authentication (MFA), and Active Directory sync.</t>
+        </is>
+      </c>
+      <c r="E64" s="9" t="inlineStr">
+        <is>
+          <t>Advanced SSO integrations pause upon trial/subscription expiry.</t>
+        </is>
+      </c>
+    </row>
+    <row r="65">
+      <c r="A65" s="4" t="inlineStr">
+        <is>
+          <t>IT &amp; Security</t>
+        </is>
+      </c>
+      <c r="B65" s="5" t="inlineStr">
+        <is>
+          <t>Zoho QEngine</t>
+        </is>
+      </c>
+      <c r="C65" s="6" t="inlineStr">
+        <is>
+          <t>15-day Free Trial only.</t>
+        </is>
+      </c>
+      <c r="D65" s="6" t="inlineStr">
+        <is>
+          <t>Test automation platform for web, mobile, and API testing with low-code test recorders.</t>
+        </is>
+      </c>
+      <c r="E65" s="6" t="inlineStr">
+        <is>
+          <t>Automated test executions pause after trial ends.</t>
         </is>
       </c>
     </row>

</xml_diff>